<commit_message>
Fix bug in calc_percent_return() and test_calc_percent_return().
</commit_message>
<xml_diff>
--- a/percent_return_on_margin.xlsx
+++ b/percent_return_on_margin.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darin\Proton Drive\darindavis\My files\Python\Projects\tradovate_orders_filled_from_tv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EF186A-19A1-419C-91C4-4A7E9774770D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7371E96F-FA98-435A-8093-781E85147488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28950" yWindow="-14880" windowWidth="13800" windowHeight="13785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24660" yWindow="-13725" windowWidth="18960" windowHeight="12075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Ticker</t>
   </si>
@@ -392,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.796875" bestFit="1" customWidth="1"/>
@@ -449,8 +449,8 @@
         <v>0.2</v>
       </c>
       <c r="G2">
-        <f>F2/10</f>
-        <v>0.02</v>
+        <f>E2/(D2/10)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
@@ -461,22 +461,22 @@
         <v>1000</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <f t="shared" si="0"/>
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="E3">
-        <v>109.5</v>
+        <v>100</v>
       </c>
       <c r="F3">
         <f t="shared" si="1"/>
-        <v>2.7375E-2</v>
+        <v>0.1</v>
       </c>
       <c r="G3">
-        <f>F3/10</f>
-        <v>2.7374999999999999E-3</v>
+        <f t="shared" ref="G3:G7" si="2">E3/(D3/10)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
@@ -501,8 +501,8 @@
         <v>0.2</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G8" si="2">F4/10</f>
-        <v>0.02</v>
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
@@ -528,7 +528,7 @@
       </c>
       <c r="G5">
         <f t="shared" si="2"/>
-        <v>0.02</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
@@ -554,7 +554,7 @@
       </c>
       <c r="G6">
         <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
@@ -580,33 +580,7 @@
       </c>
       <c r="G7">
         <f t="shared" si="2"/>
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>2000</v>
-      </c>
-      <c r="C8">
-        <v>10</v>
-      </c>
-      <c r="D8">
-        <f>B8*C8</f>
-        <v>20000</v>
-      </c>
-      <c r="E8">
-        <v>-611</v>
-      </c>
-      <c r="F8">
-        <f>E8/D8</f>
-        <v>-3.0550000000000001E-2</v>
-      </c>
-      <c r="G8">
-        <f t="shared" si="2"/>
-        <v>-3.055E-3</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>